<commit_message>
startup read data base ; fix
</commit_message>
<xml_diff>
--- a/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Powertrain.xlsx
+++ b/Scripts_Data/Data_Vehicle/sm_car_ARTTU_Powertrain.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrei/Desktop/FSAE/Vehicle Model/VehicleModel/Scripts_Data/Data_Vehicle/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280B0E4C-C3FC-2A42-B007-E177DA193841}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A2458B5-5250-044B-A5D4-803D0CC25C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7040" yWindow="720" windowWidth="17160" windowHeight="19820" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7040" yWindow="720" windowWidth="17160" windowHeight="19820" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Power" sheetId="5" r:id="rId1"/>
@@ -1117,6 +1117,9 @@
     <xf numFmtId="49" fontId="3" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1128,9 +1131,6 @@
     </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3790,7 +3790,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="90" t="s">
+      <c r="A5" s="91" t="s">
         <v>32</v>
       </c>
       <c r="B5" s="11" t="s">
@@ -3807,7 +3807,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="14" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="91"/>
+      <c r="A6" s="92"/>
       <c r="B6" s="14" t="s">
         <v>35</v>
       </c>
@@ -3822,7 +3822,7 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="92"/>
+      <c r="A7" s="93"/>
       <c r="B7" s="14" t="s">
         <v>39</v>
       </c>
@@ -3837,7 +3837,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="90" t="s">
+      <c r="A8" s="91" t="s">
         <v>41</v>
       </c>
       <c r="B8" s="11" t="s">
@@ -3854,7 +3854,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="91"/>
+      <c r="A9" s="92"/>
       <c r="B9" s="14" t="s">
         <v>35</v>
       </c>
@@ -3869,7 +3869,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="92"/>
+      <c r="A10" s="93"/>
       <c r="B10" s="14" t="s">
         <v>44</v>
       </c>
@@ -3884,7 +3884,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="91" t="s">
         <v>46</v>
       </c>
       <c r="B11" s="85" t="s">
@@ -3899,7 +3899,7 @@
       <c r="E11" s="64"/>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="91"/>
+      <c r="A12" s="92"/>
       <c r="B12" s="85" t="s">
         <v>47</v>
       </c>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="B13" s="86"/>
       <c r="C13" s="59">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="D13" s="20" t="s">
         <v>50</v>
@@ -3944,122 +3944,122 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
     <row r="1" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="94">
+      <c r="A1" s="90">
         <v>195.6</v>
       </c>
-      <c r="B1" s="94">
+      <c r="B1" s="90">
         <v>193.7</v>
       </c>
-      <c r="C1" s="94">
+      <c r="C1" s="90">
         <v>192.4</v>
       </c>
-      <c r="D1" s="94">
+      <c r="D1" s="90">
         <v>191.1</v>
       </c>
-      <c r="E1" s="94">
+      <c r="E1" s="90">
         <v>190.8</v>
       </c>
-      <c r="F1" s="94">
+      <c r="F1" s="90">
         <v>189.1</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="94">
+      <c r="A2" s="90">
         <v>187</v>
       </c>
-      <c r="B2" s="94">
+      <c r="B2" s="90">
         <v>186.4</v>
       </c>
-      <c r="C2" s="94">
+      <c r="C2" s="90">
         <v>185.2</v>
       </c>
-      <c r="D2" s="94">
+      <c r="D2" s="90">
         <v>184.8</v>
       </c>
-      <c r="E2" s="94">
+      <c r="E2" s="90">
         <v>182.4</v>
       </c>
-      <c r="F2" s="94">
+      <c r="F2" s="90">
         <v>180.9</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="94">
+      <c r="A3" s="90">
         <v>179.5</v>
       </c>
-      <c r="B3" s="94">
+      <c r="B3" s="90">
         <v>178.2</v>
       </c>
-      <c r="C3" s="94">
+      <c r="C3" s="90">
         <v>177.9</v>
       </c>
-      <c r="D3" s="94">
+      <c r="D3" s="90">
         <v>176.7</v>
       </c>
-      <c r="E3" s="94">
+      <c r="E3" s="90">
         <v>174.9</v>
       </c>
-      <c r="F3" s="94">
+      <c r="F3" s="90">
         <v>171.2</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="94">
+      <c r="A4" s="90">
         <v>169.8</v>
       </c>
-      <c r="B4" s="94">
+      <c r="B4" s="90">
         <v>168.7</v>
       </c>
-      <c r="C4" s="94">
+      <c r="C4" s="90">
         <v>166.5</v>
       </c>
-      <c r="D4" s="94">
+      <c r="D4" s="90">
         <v>164.7</v>
       </c>
-      <c r="E4" s="94">
+      <c r="E4" s="90">
         <v>161.9</v>
       </c>
-      <c r="F4" s="94">
+      <c r="F4" s="90">
         <v>161.19999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A5" s="94">
+      <c r="A5" s="90">
         <v>160.69999999999999</v>
       </c>
-      <c r="B5" s="94">
+      <c r="B5" s="90">
         <v>159.4</v>
       </c>
-      <c r="C5" s="94">
+      <c r="C5" s="90">
         <v>158.6</v>
       </c>
-      <c r="D5" s="94">
+      <c r="D5" s="90">
         <v>157.5</v>
       </c>
-      <c r="E5" s="94">
+      <c r="E5" s="90">
         <v>156.9</v>
       </c>
-      <c r="F5" s="94">
+      <c r="F5" s="90">
         <v>155.19999999999999</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A6" s="94">
+      <c r="A6" s="90">
         <v>154.80000000000001</v>
       </c>
-      <c r="B6" s="94">
+      <c r="B6" s="90">
         <v>153.69999999999999</v>
       </c>
-      <c r="C6" s="94">
+      <c r="C6" s="90">
         <v>152.4</v>
       </c>
-      <c r="D6" s="94">
+      <c r="D6" s="90">
         <v>151.69999999999999</v>
       </c>
-      <c r="E6" s="94">
+      <c r="E6" s="90">
         <v>150.30000000000001</v>
       </c>
-      <c r="F6" s="94">
+      <c r="F6" s="90">
         <v>148.80000000000001</v>
       </c>
     </row>
@@ -4074,122 +4074,122 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
     <row r="1" spans="1:6" ht="13" x14ac:dyDescent="0.15">
-      <c r="A1" s="94">
+      <c r="A1" s="90">
         <v>4.2300000000000003E-3</v>
       </c>
-      <c r="B1" s="94">
+      <c r="B1" s="90">
         <v>3.8E-3</v>
       </c>
-      <c r="C1" s="94">
+      <c r="C1" s="90">
         <v>3.7699999999999999E-3</v>
       </c>
-      <c r="D1" s="94">
+      <c r="D1" s="90">
         <v>3.6600000000000001E-3</v>
       </c>
-      <c r="E1" s="94">
+      <c r="E1" s="90">
         <v>3.62E-3</v>
       </c>
-      <c r="F1" s="94">
+      <c r="F1" s="90">
         <v>3.5899999999999999E-3</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="94">
+      <c r="A2" s="90">
         <v>3.5699999999999998E-3</v>
       </c>
-      <c r="B2" s="94">
+      <c r="B2" s="90">
         <v>3.2699999999999999E-3</v>
       </c>
-      <c r="C2" s="94">
+      <c r="C2" s="90">
         <v>3.1900000000000001E-3</v>
       </c>
-      <c r="D2" s="94">
+      <c r="D2" s="90">
         <v>3.8E-3</v>
       </c>
-      <c r="E2" s="94">
+      <c r="E2" s="90">
         <v>3.13E-3</v>
       </c>
-      <c r="F2" s="94">
+      <c r="F2" s="90">
         <v>3.0799999999999998E-3</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="94">
+      <c r="A3" s="90">
         <v>3.15E-3</v>
       </c>
-      <c r="B3" s="94">
+      <c r="B3" s="90">
         <v>2.98E-3</v>
       </c>
-      <c r="C3" s="94">
+      <c r="C3" s="90">
         <v>3.0999999999999999E-3</v>
       </c>
-      <c r="D3" s="94">
+      <c r="D3" s="90">
         <v>2.8E-3</v>
       </c>
-      <c r="E3" s="94">
+      <c r="E3" s="90">
         <v>2.7699999999999999E-3</v>
       </c>
-      <c r="F3" s="94">
+      <c r="F3" s="90">
         <v>2.7499999999999998E-3</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="94">
+      <c r="A4" s="90">
         <v>2.7699999999999999E-3</v>
       </c>
-      <c r="B4" s="94">
+      <c r="B4" s="90">
         <v>2.8800000000000002E-3</v>
       </c>
-      <c r="C4" s="94">
+      <c r="C4" s="90">
         <v>3.1099999999999999E-3</v>
       </c>
-      <c r="D4" s="94">
+      <c r="D4" s="90">
         <v>3.2399999999999998E-3</v>
       </c>
-      <c r="E4" s="94">
+      <c r="E4" s="90">
         <v>3.0999999999999999E-3</v>
       </c>
-      <c r="F4" s="94">
+      <c r="F4" s="90">
         <v>2.7299999999999998E-3</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="94">
+      <c r="A5" s="90">
         <v>3.3E-3</v>
       </c>
-      <c r="B5" s="94">
+      <c r="B5" s="90">
         <v>2.8900000000000002E-3</v>
       </c>
-      <c r="C5" s="94">
+      <c r="C5" s="90">
         <v>2.9399999999999999E-3</v>
       </c>
-      <c r="D5" s="94">
+      <c r="D5" s="90">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="E5" s="94">
+      <c r="E5" s="90">
         <v>2.9299999999999999E-3</v>
       </c>
-      <c r="F5" s="94">
+      <c r="F5" s="90">
         <v>2.8800000000000002E-3</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="94">
+      <c r="A6" s="90">
         <v>2.9399999999999999E-3</v>
       </c>
-      <c r="B6" s="94">
+      <c r="B6" s="90">
         <v>3.29E-3</v>
       </c>
-      <c r="C6" s="94">
+      <c r="C6" s="90">
         <v>3.1199999999999999E-3</v>
       </c>
-      <c r="D6" s="94">
+      <c r="D6" s="90">
         <v>2.7299999999999998E-3</v>
       </c>
-      <c r="E6" s="94">
+      <c r="E6" s="90">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="F6" s="94">
+      <c r="F6" s="90">
         <v>2.3999999999999998E-3</v>
       </c>
     </row>
@@ -4255,7 +4255,7 @@
       <c r="E4" s="10"/>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="90" t="s">
+      <c r="A5" s="91" t="s">
         <v>51</v>
       </c>
       <c r="B5" s="47" t="s">
@@ -4270,7 +4270,7 @@
       <c r="E5" s="22"/>
     </row>
     <row r="6" spans="1:5" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="93"/>
+      <c r="A6" s="94"/>
       <c r="B6" s="48" t="s">
         <v>55</v>
       </c>
@@ -4296,7 +4296,7 @@
       <c r="E7" s="81"/>
     </row>
     <row r="8" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="90" t="s">
+      <c r="A8" s="91" t="s">
         <v>59</v>
       </c>
       <c r="B8" s="49" t="s">
@@ -4311,7 +4311,7 @@
       <c r="E8" s="45"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="91"/>
+      <c r="A9" s="92"/>
       <c r="B9" s="50" t="s">
         <v>55</v>
       </c>
@@ -4324,7 +4324,7 @@
       <c r="E9" s="23"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="93"/>
+      <c r="A10" s="94"/>
       <c r="B10" s="61" t="s">
         <v>28</v>
       </c>
@@ -4337,7 +4337,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="90" t="s">
+      <c r="A11" s="91" t="s">
         <v>60</v>
       </c>
       <c r="B11" s="65" t="s">
@@ -4352,7 +4352,7 @@
       <c r="E11" s="68"/>
     </row>
     <row r="12" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="91"/>
+      <c r="A12" s="92"/>
       <c r="B12" s="69" t="s">
         <v>63</v>
       </c>
@@ -4365,7 +4365,7 @@
       <c r="E12" s="72"/>
     </row>
     <row r="13" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="91"/>
+      <c r="A13" s="92"/>
       <c r="B13" s="69" t="s">
         <v>28</v>
       </c>
@@ -4378,7 +4378,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="91"/>
+      <c r="A14" s="92"/>
       <c r="B14" s="69" t="s">
         <v>64</v>
       </c>
@@ -4391,7 +4391,7 @@
       <c r="E14" s="72"/>
     </row>
     <row r="15" spans="1:5" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="93"/>
+      <c r="A15" s="94"/>
       <c r="B15" s="73" t="s">
         <v>66</v>
       </c>
@@ -5648,6 +5648,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="9557458c-24b5-4c97-84ed-4c402655f54f">
@@ -5656,15 +5665,6 @@
     <TaxCatchAll xmlns="72e3c584-9879-4b35-b9d8-6a248c93e240" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5687,6 +5687,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8192A017-E4B6-4D7F-8544-3BE30BB952E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3314153-DE99-46E1-9177-E565F1EC3082}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -5695,12 +5703,4 @@
     <ds:schemaRef ds:uri="72e3c584-9879-4b35-b9d8-6a248c93e240"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8192A017-E4B6-4D7F-8544-3BE30BB952E0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>